<commit_message>
Record author's answers to submission worksheet items (30 Sep 2026)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KoT3i8geZspYBMMKVYJUTG
</commit_message>
<xml_diff>
--- a/docs/thesis/Thesis_Submission_Worksheet_to_15Oct2026.xlsx
+++ b/docs/thesis/Thesis_Submission_Worksheet_to_15Oct2026.xlsx
@@ -612,10 +612,14 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>30 Sep: rule = after a failure or game over, a player who never played again is a dropout; one who played again returned. Measured before zero-failure was implemented. To confirm: did Stage-3A players first play a version with game over? How does this relate to the '5 attempts' label?</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -653,10 +657,14 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>30 Sep: players answered by themselves right after playing, at the point they decided to stop. Still to confirm: only D1 and D2? 1–5 scale? language? wording as in the FOR_REVIEW draft?</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -694,10 +702,14 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>30 Sep: two figures = whole cohort 112/120 = 93.3%; ages 65–80 35/41 = 85.4%. Decision with Prof. Cheung still open.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -735,10 +747,14 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>30 Sep: nothing new needed. Claude to cite the Stage-2 files on record instead of FRA_Raw_Data_N30.xlsx.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -776,10 +792,14 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>30 Sep: author collecting therapists' summary photocopies from the Guangzhou centre next week.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -817,10 +837,14 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>30 Sep: F4 explained (top FIAS category = observed non-return; six players scoring 9–10, all among the eight one-session players). Author sorting out.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -858,10 +882,14 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>30 Sep: play recorded at the centre in handwritten logs. Awaiting confirmation that the game software's electronic session and AI-call records were not kept.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -899,10 +927,14 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr"/>
+          <t>Cannot supply</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>30 Sep: author decision — no ethics clarification sought (thesis makes no Stage-3B claim). Thesis keeps the scope as a stated open item.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -940,10 +972,14 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>30 Sep: waiting for Prof. Cheung's reply.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">

</xml_diff>

<commit_message>
Thesis V52 and Paper 3 R12: author's answers on dropout rule, questionnaire, Stage-2 files and logs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KoT3i8geZspYBMMKVYJUTG
</commit_message>
<xml_diff>
--- a/docs/thesis/Thesis_Submission_Worksheet_to_15Oct2026.xlsx
+++ b/docs/thesis/Thesis_Submission_Worksheet_to_15Oct2026.xlsx
@@ -571,10 +571,14 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>30 Sep: V52 now says the logbook claim is pending the 120 returned files — author has not yet answered; Claude will lower the claim if the files cannot be sent.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -612,12 +616,12 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>30 Sep: rule = after a failure or game over, a player who never played again is a dropout; one who played again returned. Measured before zero-failure was implemented. To confirm: did Stage-3A players first play a version with game over? How does this relate to the '5 attempts' label?</t>
+          <t>V52 §6.4: failure-then-stop rule; earlier game-over version reached some players, unrecorded.</t>
         </is>
       </c>
     </row>
@@ -662,7 +666,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>30 Sep: players answered by themselves right after playing, at the point they decided to stop. Still to confirm: only D1 and D2? 1–5 scale? language? wording as in the FOR_REVIEW draft?</t>
+          <t>V52 App D: two items, 1–5, 4–5 positive, answered right after play. OPEN: summary labels ("eye-leg coordination"; "regular health training if accessible") differ from App D wording — confirm which wording players saw.</t>
         </is>
       </c>
     </row>
@@ -702,12 +706,12 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>30 Sep: two figures = whole cohort 112/120 = 93.3%; ages 65–80 35/41 = 85.4%. Decision with Prof. Cheung still open.</t>
+          <t>Author decision: keep 93.3% and 85.4%.</t>
         </is>
       </c>
     </row>
@@ -747,12 +751,12 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>30 Sep: nothing new needed. Claude to cite the Stage-2 files on record instead of FRA_Raw_Data_N30.xlsx.</t>
+          <t>V52 cites stage2_clean.csv, FRA_32 data set, Stage-2 logbook.</t>
         </is>
       </c>
     </row>
@@ -842,7 +846,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>30 Sep: F4 explained (top FIAS category = observed non-return; six players scoring 9–10, all among the eight one-session players). Author sorting out.</t>
+          <t>Author: F4 identified from after-game interview records kept at the centre; records to be collected. Reconcile with Appendix C (F4 interview "designed, not administered").</t>
         </is>
       </c>
     </row>
@@ -882,12 +886,12 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>30 Sep: play recorded at the centre in handwritten logs. Awaiting confirmation that the game software's electronic session and AI-call records were not kept.</t>
+          <t>V52 §8.9 and G.2: play recorded by hand; software logs not kept.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Worksheet: F4 correction, D1/D2 stage question, logbook files clarification
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KoT3i8geZspYBMMKVYJUTG
</commit_message>
<xml_diff>
--- a/docs/thesis/Thesis_Submission_Worksheet_to_15Oct2026.xlsx
+++ b/docs/thesis/Thesis_Submission_Worksheet_to_15Oct2026.xlsx
@@ -576,7 +576,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>30 Sep: V52 now says the logbook claim is pending the 120 returned files — author has not yet answered; Claude will lower the claim if the files cannot be sent.</t>
+          <t>30 Sep: author asked whether all 120 e-mails are needed. Answer: only the returned result files and answers, not the e-mails; or Claude lowers the claim.</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>V52 App D: two items, 1–5, 4–5 positive, answered right after play. OPEN: summary labels ("eye-leg coordination"; "regular health training if accessible") differ from App D wording — confirm which wording players saw.</t>
+          <t>V52 App D: two items, 1–5, 4–5 positive, answered right after play. OPEN: summary labels ("eye-leg coordination"; "regular health training if accessible") differ from App D wording — confirm which wording players saw. | 30 Sep: author thought D1 was Stage 2 and D2 Stage 3; record shows both items in the Stage-3 summary (86/120, 76/120) and no coordination item in the Stage-2 nine-question form. Author to re-check.</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Author: F4 identified from after-game interview records kept at the centre; records to be collected. Reconcile with Appendix C (F4 interview "designed, not administered").</t>
+          <t>CORRECTED 30 Sep: author confirms F4 = players who lost interest after the first attempt; an interview was designed for them but none was given (matches Appendix C). Still needed: the six IDs and the scoring rule, or withdraw Figure 5.6 and the composite scores.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Worksheet: D1 purpose, F4 IDs found, logbook files
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KoT3i8geZspYBMMKVYJUTG
</commit_message>
<xml_diff>
--- a/docs/thesis/Thesis_Submission_Worksheet_to_15Oct2026.xlsx
+++ b/docs/thesis/Thesis_Submission_Worksheet_to_15Oct2026.xlsx
@@ -576,7 +576,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>30 Sep: author asked whether all 120 e-mails are needed. Answer: only the returned result files and answers, not the e-mails; or Claude lowers the claim.</t>
+          <t>30 Sep: author asked whether all 120 e-mails are needed. Answer: only the returned result files and answers, not the e-mails; or Claude lowers the claim. | Confirmed to author: all 120 result files are needed for the reconciliation claim; otherwise lower the claim.</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>V52 App D: two items, 1–5, 4–5 positive, answered right after play. OPEN: summary labels ("eye-leg coordination"; "regular health training if accessible") differ from App D wording — confirm which wording players saw. | 30 Sep: author thought D1 was Stage 2 and D2 Stage 3; record shows both items in the Stage-3 summary (86/120, 76/120) and no coordination item in the Stage-2 nine-question form. Author to re-check.</t>
+          <t>V52 App D: two items, 1–5, 4–5 positive, answered right after play. OPEN: summary labels ("eye-leg coordination"; "regular health training if accessible") differ from App D wording — confirm which wording players saw. | 30 Sep: author thought D1 was Stage 2 and D2 Stage 3; record shows both items in the Stage-3 summary (86/120, 76/120) and no coordination item in the Stage-2 nine-question form. Author to re-check. | 30 Sep (later): author confirms D1 is Stage 3; purpose = check whether players saw the game as exercising the eye-leg coordination the FRA measures. To add to Appendix D in next pass. Exact wording as sent still not supplied.</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>CORRECTED 30 Sep: author confirms F4 = players who lost interest after the first attempt; an interview was designed for them but none was given (matches Appendix C). Still needed: the six IDs and the scoring rule, or withdraw Figure 5.6 and the composite scores.</t>
+          <t>CORRECTED 30 Sep: author confirms F4 = players who lost interest after the first attempt; an interview was designed for them but none was given (matches Appendix C). Still needed: the six IDs and the scoring rule, or withdraw Figure 5.6 and the composite scores. | 30 Sep (later): author has found the six IDs; awaiting them.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Flag: archived 'Stage 3' game v2.2 was created 13 Jul 2026, not the Mar-Apr Stage-3A build
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KoT3i8geZspYBMMKVYJUTG
</commit_message>
<xml_diff>
--- a/docs/thesis/Thesis_Submission_Worksheet_to_15Oct2026.xlsx
+++ b/docs/thesis/Thesis_Submission_Worksheet_to_15Oct2026.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1517,6 +1517,51 @@
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>1 Must</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>§6.4 (thesis); Game Build and Data Availability (Paper 3)</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Paper 3 names Alpine_Coordination_Game_Stage3_v2.2.html as the archived Stage 3A build and describes its features; thesis §6.4 (V52) refers to 'the archived build with its zero-failure mode'.</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Repository history: that file was created on 13 July 2026 ('Redesign Stage-3 game', v2 → v2.2 the same day), after the March–April study. The game actually sent to players in March–April is not in the repository.</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>The HTML game file your research assistants sent to players in March–April (an e-mail attachment or the file on the prepared iPads), plus the earlier version with game over if it still exists.</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Claude corrects Paper 3 and §6.4: the build as distributed is not archived; the July 2026 file is a later redesign and its features are not evidence of what Stage 3A players used.</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>30 Sep: found when the author asked for the March–April game.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:I24"/>

</xml_diff>

<commit_message>
Archive Stage 3 Research Build v1.0 found by author; document builds and batch-file consequence
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KoT3i8geZspYBMMKVYJUTG
</commit_message>
<xml_diff>
--- a/docs/thesis/Thesis_Submission_Worksheet_to_15Oct2026.xlsx
+++ b/docs/thesis/Thesis_Submission_Worksheet_to_15Oct2026.xlsx
@@ -1554,12 +1554,12 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>30 Sep: found when the author asked for the March–April game.</t>
+          <t>30 Sep: found when the author asked for the March–April game. | 30 Sep: author found 'Alpine_Coordination_Game_Stage31.html' = STAGE 3 RESEARCH BUILD v1.0 (not in repo history); archived. To confirm: where found, file date, and that it was sent to players from April. Then Claude rewrites Paper 3 build description and §6.4.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Submission plan 1-15 Oct 2026 (schedule, task cards, templates, PolyU format check); tracker schedule sheet and gate items
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KoT3i8geZspYBMMKVYJUTG
</commit_message>
<xml_diff>
--- a/docs/thesis/Thesis_Submission_Worksheet_to_15Oct2026.xlsx
+++ b/docs/thesis/Thesis_Submission_Worksheet_to_15Oct2026.xlsx
@@ -7,16 +7,15 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 Records from you" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 Claude will fix" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 Final production" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4 Plan to 15 Oct" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4 Schedule 1-15 Oct" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 Records from you" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 Claude will fix" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 Final production" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'1 Records from you'!$A$1:$I$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2 Claude will fix'!$A$1:$F$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'3 Final production'!$A$1:$E$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'4 Plan to 15 Oct'!$A$1:$B$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'1 Records from you'!$A$1:$I$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'2 Claude will fix'!$A$1:$F$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'3 Final production'!$A$1:$E$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -25,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,6 +35,9 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="6">
@@ -92,7 +94,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -107,6 +109,10 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -474,7 +480,680 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:E25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Who</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Task</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>Plan card / template</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Thu 1 Oct</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>You</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Send T1 to the EngD Programme Office</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>A1 / T1</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Thu 1 Oct</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>You</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Send T2 to Prof. Cheung (meeting request)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>A2 / T2</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Thu 1 Oct</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>You</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Send T3 to the research assistant</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>B1 / T3</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Thu 1 Oct</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>You</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Reply to Claude: game picture, where/when v1.0 was found; invitation date line</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>B2, B3</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Fri 2 Oct</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>You</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Phone the Programme Office if no reply; book Prof. Cheung meeting; ask about Turnitin access</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>A1, A2, A3</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Fri 2 Oct</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Apply game and invitation answers; decide Figure 1</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>B2, B3</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Sat 3–Sun 4 Oct</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>You</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Confirm T7 (AI use) and T8 (acknowledgements); write T5 statement for D01, D13, BYXXMT; send T6 to Dr Choy and Dr Lau</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>A4, B4, B7</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Sat 3–Sun 4 Oct</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Draft Appendix G manifest and build-lineage rows</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Claude list 5</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Mon 5–Tue 6 Oct</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>You</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Send T4 to the Guangzhou centre; collect copies; ask for the video consent; remind the research assistant</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>B5, B6</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Mon 5–Tue 6 Oct</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Insert T7/T8; add expert replies</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Wed 7 Oct</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>You</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Research assistant deadline: Stage 3 records (partial is fine) and questionnaire as sent</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>B1, B8</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Thu 8 Oct</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>CHECKPOINT 1: add Stage 3 records or apply prepared wording; update §6.4, Chapter 6, Paper 3</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Fri 9 Oct</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>You</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>All other records due; send Prof. Cheung the reading copy</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>B4–B9, A2</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Fri 9 Oct</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>CHECKPOINT 2: apply fallbacks; produce reading copy and one-page change summary</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Sat 10–Sun 11 Oct</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>You</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Read the whole thesis with checklist T9; send corrections</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>T9</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Sat 10–Sun 11 Oct</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Independent consistency check of the whole thesis</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Mon 12 Oct</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>You</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Run the similarity report; collect Prof. Cheung's comments</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Mon 12 Oct</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Apply your and Prof. Cheung's corrections</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr"/>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>You</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Fill in forms (approval, AI declaration, intention to submit)</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>A1, A4</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Tue 13 Oct</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>CHECKPOINT 3: final production and PDF draft</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Group C</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Wed 14 Oct</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>You</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Prof. Cheung signs; send Stage 3B files received today (count closes 23:59)</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Wed 14 Oct</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Enter final Stage 3B count; final PDF</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr"/>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Thu 15 Oct</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>You</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Submit PDF and forms; keep the receipt</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Thu 15 Oct</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Archive the submitted version with checksum</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr"/>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="E2:E25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Not started,Done,Late"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -576,7 +1255,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>30 Sep: author asked whether all 120 e-mails are needed. Answer: only the returned result files and answers, not the e-mails; or Claude lowers the claim. | Confirmed to author: all 120 result files are needed for the reconciliation claim; otherwise lower the claim. | 30 Sep: author reports the Stage-3 returns arrived in mixed formats (some CSV, some text in e-mails), not organised at the time; asking the research assistant who handled collection. Send as-is; Claude will organise. | 30 Sep: author's 'Stage_3_game_telemetry.xlsx' checked — it is a copy of the synthetic demo data (TEST-001…TEST-120; 569/569 rows match), NOT usable; archived under SYNTHETIC_copies_received/. | 30 Sep: author expects RAs did not keep all files but have records, especially for the 65–80 players. Plan: RAs fill the template for whoever has records; thesis reports coverage (n of 120, by band) and whether that subset matches the summary; aggregate summary stays the source for all 120.</t>
+          <t>DUE: Due Wed 7 Oct (RA); decision Thu 8 Oct | 30 Sep: author asked whether all 120 e-mails are needed. Answer: only the returned result files and answers, not the e-mails; or Claude lowers the claim. | Confirmed to author: all 120 result files are needed for the reconciliation claim; otherwise lower the claim. | 30 Sep: author reports the Stage-3 returns arrived in mixed formats (some CSV, some text in e-mails), not organised at the time; asking the research assistant who handled collection. Send as-is; Claude will organise. | 30 Sep: author's 'Stage_3_game_telemetry.xlsx' checked — it is a copy of the synthetic demo data (TEST-001…TEST-120; 569/569 rows match), NOT usable; archived under SYNTHETIC_copies_received/. | 30 Sep: author expects RAs did not keep all files but have records, especially for the 65–80 players. Plan: RAs fill the template for whoever has records; thesis reports coverage (n of 120, by band) and whether that subset matches the summary; aggregate summary stays the source for all 120.</t>
         </is>
       </c>
     </row>
@@ -666,7 +1345,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>V52 App D: two items, 1–5, 4–5 positive, answered right after play. OPEN: summary labels ("eye-leg coordination"; "regular health training if accessible") differ from App D wording — confirm which wording players saw. | 30 Sep: author thought D1 was Stage 2 and D2 Stage 3; record shows both items in the Stage-3 summary (86/120, 76/120) and no coordination item in the Stage-2 nine-question form. Author to re-check. | 30 Sep (later): author confirms D1 is Stage 3; purpose = check whether players saw the game as exercising the eye-leg coordination the FRA measures. To add to Appendix D in next pass. Exact wording as sent still not supplied.</t>
+          <t>DUE: Due Wed 7 Oct | V52 App D: two items, 1–5, 4–5 positive, answered right after play. OPEN: summary labels ("eye-leg coordination"; "regular health training if accessible") differ from App D wording — confirm which wording players saw. | 30 Sep: author thought D1 was Stage 2 and D2 Stage 3; record shows both items in the Stage-3 summary (86/120, 76/120) and no coordination item in the Stage-2 nine-question form. Author to re-check. | 30 Sep (later): author confirms D1 is Stage 3; purpose = check whether players saw the game as exercising the eye-leg coordination the FRA measures. To add to Appendix D in next pass. Exact wording as sent still not supplied.</t>
         </is>
       </c>
     </row>
@@ -801,7 +1480,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>30 Sep: author collecting therapists' summary photocopies from the Guangzhou centre next week.</t>
+          <t>DUE: Due Fri 9 Oct (centre copies) | 30 Sep: author collecting therapists' summary photocopies from the Guangzhou centre next week.</t>
         </is>
       </c>
     </row>
@@ -846,7 +1525,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>30 Sep: F4 = S2-P006, P007, P011, P015, P026, P028 (author; V54's P027/P029 were wrong, corrected in V55). All one session; 006/007/015 improved; 015 is the unverified record. Scoring rule (0–10) still outstanding.</t>
+          <t>DUE: Scoring rule optional — fallback already in text | 30 Sep: F4 = S2-P006, P007, P011, P015, P026, P028 (author; V54's P027/P029 were wrong, corrected in V55). All one session; 006/007/015 improved; 015 is the unverified record. Scoring rule (0–10) still outstanding.</t>
         </is>
       </c>
     </row>
@@ -981,7 +1660,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>30 Sep: waiting for Prof. Cheung's reply.</t>
+          <t>DUE: Meeting by 9 Oct; signature Wed 14 Oct | 30 Sep: waiting for Prof. Cheung's reply.</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1703,11 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DUE: Claude drafts by 4 Oct; you check | </t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1065,7 +1748,11 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DUE: Claude drafts by 4 Oct; you check | </t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1106,7 +1793,11 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DUE: Optional; due Fri 9 Oct | </t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -1147,7 +1838,11 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DUE: Optional; due Fri 9 Oct | </t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1188,7 +1883,11 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DUE: Optional; due Fri 9 Oct | </t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -1229,7 +1928,11 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr"/>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DUE: Due Fri 9 Oct (T6) | </t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1270,7 +1973,11 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DUE: Due Fri 9 Oct | </t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1311,7 +2018,11 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DUE: Claude by 9 Oct | </t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1352,7 +2063,11 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DUE: Optional; one line by 9 Oct | </t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -1393,7 +2108,11 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr"/>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DUE: Statement (T5) by Sun 4 Oct; files until 14 Oct 23:59 | </t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -1434,7 +2153,11 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="I22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DUE: Optional; due Fri 9 Oct | </t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -1475,7 +2198,11 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="I23" s="2" t="inlineStr"/>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DUE: Your OK any time | </t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -1516,7 +2243,11 @@
           <t>Not started</t>
         </is>
       </c>
-      <c r="I24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DUE: Check by Fri 9 Oct | </t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -1559,14 +2290,242 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>30 Sep: found when the author asked for the March–April game. | 30 Sep: author found 'Alpine_Coordination_Game_Stage31.html' = STAGE 3 RESEARCH BUILD v1.0 (not in repo history); archived. To confirm: where found, file date, and that it was sent to players from April. Then Claude rewrites Paper 3 build description and §6.4.</t>
+          <t>DUE: Answers due Fri 2 Oct (plan card B2) | 30 Sep: found when the author asked for the March–April game. | 30 Sep: author found 'Alpine_Coordination_Game_Stage31.html' = STAGE 3 RESEARCH BUILD v1.0 (not in repo history); archived. To confirm: where found, file date, and that it was sent to players from April. Then Claude rewrites Paper 3 build description and §6.4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>1 Must</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Submission (external gate G1)</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>The EngD page says the thesis is submitted with an "Intention to submit thesis form". For MPhil/PhD, Form GSB/2B needs at least 4 months' notice.</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Not known whether the EngD has the same notice rule, or whether your form was filed.</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Send plan template T1 to feng.engd@polyu.edu.hk; telephone on 2 Oct if no reply.</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>If notice was needed and not given, the submission date moves; the thesis stays ready.</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Due Fri 2 Oct</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>1 Must</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Approval form (external gate G3)</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>The supervisor's approval form records a similarity (Turnitin) percentage with his comment.</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>No similarity report yet.</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Ask how to get Turnitin access (T1/T2); run it on 12 Oct on the reading copy; send me the report.</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Ask the Programme Office to run it.</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>Due Mon 12 Oct</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>1 Must</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Front matter; approval form (gate G4)</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>The approval form asks whether generative AI was used to prepare the thesis (Honour Declaration Form). The thesis declares AI only for game development (§5.3.9).</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>No declaration for AI help with writing, revision and checking.</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Correct and confirm plan template T7; I insert it. Complete the Honour Declaration Form.</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Do not submit without it.</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Due Fri 9 Oct</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>2 Should</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Acknowledgements (format rule)</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>PolyU rules: contributions by others are declared in the Acknowledgements.</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Research assistants and therapists' summary work not acknowledged.</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Confirm plan template T8; I insert it.</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>I insert T8 as written if you have no changes.</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>Due Fri 9 Oct</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>2 Should</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Front pages (format rule)</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>PolyU rules require a cover page (title and name in capitals, degree, university, year of award) before the title page.</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>V58 has one combined title page with a "Thesis Title" label.</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Nothing, unless the Programme Office sends an EngD template — forward it to me.</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>I build the cover page to the Graduate School rules on 13 Oct.</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>Claude, 13 Oct</t>
         </is>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:I24"/>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation sqref="H2:H24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Not started,In progress,Sent to Claude,Done,Cannot supply"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H25:H30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not started,In progress,Sent to Claude,Done,Cannot supply"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1574,13 +2533,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1839,6 +2798,66 @@
       </c>
       <c r="F9" s="2" t="inlineStr"/>
     </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Cut the abstract to 496 words (PolyU limit 200–500) and change "desktop game" to "browser game".</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Abstract</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Done in thesis V58 (1 Oct)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Insert the AI declaration (T7) and acknowledgements (T8) once you confirm them; build the cover page; rebuild contents and lists from the final PDF; build the text-searchable PDF.</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Front matter; whole thesis</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Yes: T7, T8, Programme Office reply</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>13–14 Oct</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:F9"/>
   <dataValidations count="1">
@@ -1850,7 +2869,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2028,119 +3047,4 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="110" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Dates</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Focus</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>1–3 Oct</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Send Prof. Cheung this list and the retention question (item 4). E-mail the DRC/HSESC about Stage-3B scope (item 9). Collect the Stage-3 returned CSV files (items 1–3).</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>4–7 Oct</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Items 5–8 (Stage-2 records, FIAS codebook or withdraw Figure 5.6, telemetry and logs). Claude applies fixes and fallbacks as items close.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>8–10 Oct</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Items 11–21. Claude drafts G.0 and runs a full consistency check on the new version.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>11–13 Oct</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Supervisor reads the near-final version. Final production steps 1–4.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>14 Oct</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Stage 3B: enter every return received so far. Decide whether returns arriving on 15 Oct itself can still be entered (see note).</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>15 Oct</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Submit.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>The Stage 3B cut-off and the submission are the same day. Returns arriving on 15 Oct leave almost no time to enter and check. Consider closing the thesis count at the end of 14 Oct, or submit late on 15 Oct after a final update.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:B8"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Thesis V59: Stage-3 results stated as the July 2026 aggregate summary; mixed-format returns; no participant-level compilation (numbers unchanged)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KoT3i8geZspYBMMKVYJUTG
</commit_message>
<xml_diff>
--- a/docs/thesis/Thesis_Submission_Worksheet_to_15Oct2026.xlsx
+++ b/docs/thesis/Thesis_Submission_Worksheet_to_15Oct2026.xlsx
@@ -1250,12 +1250,12 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>DUE: Due Wed 7 Oct (RA); decision Thu 8 Oct | 30 Sep: author asked whether all 120 e-mails are needed. Answer: only the returned result files and answers, not the e-mails; or Claude lowers the claim. | Confirmed to author: all 120 result files are needed for the reconciliation claim; otherwise lower the claim. | 30 Sep: author reports the Stage-3 returns arrived in mixed formats (some CSV, some text in e-mails), not organised at the time; asking the research assistant who handled collection. Send as-is; Claude will organise. | 30 Sep: author's 'Stage_3_game_telemetry.xlsx' checked — it is a copy of the synthetic demo data (TEST-001…TEST-120; 569/569 rows match), NOT usable; archived under SYNTHETIC_copies_received/. | 30 Sep: author expects RAs did not keep all files but have records, especially for the 65–80 players. Plan: RAs fill the template for whoever has records; thesis reports coverage (n of 120, by band) and whether that subset matches the summary; aggregate summary stays the source for all 120. | 1 Oct: files from RA 'Rudy' checked — both DERIVED FROM THE SYNTHETIC DATA (569/569 sessions transformed; 120/120 players' answers and demographics identical). NOT usable; archived under SYNTHETIC_copies_received/. Fallback wording recommended.</t>
+          <t>DUE: Due Wed 7 Oct (RA); decision Thu 8 Oct | 30 Sep: author asked whether all 120 e-mails are needed. Answer: only the returned result files and answers, not the e-mails; or Claude lowers the claim. | Confirmed to author: all 120 result files are needed for the reconciliation claim; otherwise lower the claim. | 30 Sep: author reports the Stage-3 returns arrived in mixed formats (some CSV, some text in e-mails), not organised at the time; asking the research assistant who handled collection. Send as-is; Claude will organise. | 30 Sep: author's 'Stage_3_game_telemetry.xlsx' checked — it is a copy of the synthetic demo data (TEST-001…TEST-120; 569/569 rows match), NOT usable; archived under SYNTHETIC_copies_received/. | 30 Sep: author expects RAs did not keep all files but have records, especially for the 65–80 players. Plan: RAs fill the template for whoever has records; thesis reports coverage (n of 120, by band) and whether that subset matches the summary; aggregate summary stays the source for all 120. | 1 Oct: files from RA 'Rudy' checked — both DERIVED FROM THE SYNTHETIC DATA (569/569 sessions transformed; 120/120 players' answers and demographics identical). NOT usable; archived under SYNTHETIC_copies_received/. Fallback wording recommended. | 1 Oct: author approved fallback; applied in V59 (claim level lowered, every number unchanged). If Rudy's original handwritten records arrive by 9 Oct (scans + dated note), Claude adds one sentence on the subset they cover.</t>
         </is>
       </c>
     </row>

</xml_diff>